<commit_message>
1. Remove SR scalar that was being applied in sim inputs - it was not really achieving the desired result. profit up ~5k. 2. Pass in SRW. SRW has impact of lwc in sgen which impacts stubble category proportions. profit up 3k 3. fix animal age in sim inputs +3k profit due to improvements to fodder. 4.pass in lambing date of the ewe themselves. 1k profit down
</commit_message>
<xml_diff>
--- a/ExcelInputs/stubble sim.xlsx
+++ b/ExcelInputs/stubble sim.xlsx
@@ -345,1732 +345,1732 @@
   <sheetData>
     <row r="1" spans="1:57">
       <c r="A1">
-        <v>0.0335925515058287</v>
+        <v>0.04261855969762757</v>
       </c>
       <c r="B1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="C1">
-        <v>0.0335925515058287</v>
+        <v>0.04261855969762757</v>
       </c>
       <c r="D1">
-        <v>0.0335925515058287</v>
+        <v>0.04261855969762757</v>
       </c>
       <c r="E1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="F1">
-        <v>0.0335925515058287</v>
+        <v>0.04261855969762757</v>
       </c>
       <c r="G1">
-        <v>0.00415337319317881</v>
+        <v>0.0441170780966807</v>
       </c>
       <c r="H1">
-        <v>0.0001530185286095631</v>
+        <v>0.004131215711950811</v>
       </c>
       <c r="I1">
-        <v>0.00415337319317881</v>
+        <v>0.0441170780966807</v>
       </c>
       <c r="J1">
-        <v>0.01080129330867494</v>
+        <v>0.03220320498910477</v>
       </c>
       <c r="K1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="L1">
-        <v>0.01080129330867494</v>
+        <v>0.03220320498910477</v>
       </c>
       <c r="M1">
-        <v>0.00415337319317881</v>
+        <v>0.0441170780966807</v>
       </c>
       <c r="N1">
-        <v>0.0001530185286095631</v>
+        <v>0.004131215711950811</v>
       </c>
       <c r="O1">
-        <v>0.00415337319317881</v>
+        <v>0.0441170780966807</v>
       </c>
       <c r="P1">
-        <v>0.00415337319317881</v>
+        <v>0.0441170780966807</v>
       </c>
       <c r="Q1">
-        <v>0.0001530185286095631</v>
+        <v>0.004131215711950811</v>
       </c>
       <c r="R1">
-        <v>0.00415337319317881</v>
+        <v>0.0441170780966807</v>
       </c>
       <c r="S1">
-        <v>0.00415337319317881</v>
+        <v>0.0441170780966807</v>
       </c>
       <c r="T1">
-        <v>0.0001530185286095631</v>
+        <v>0.004131215711950811</v>
       </c>
       <c r="U1">
-        <v>0.00415337319317881</v>
+        <v>0.0441170780966807</v>
       </c>
       <c r="V1">
-        <v>0.00415337319317881</v>
+        <v>0.0441170780966807</v>
       </c>
       <c r="W1">
-        <v>0.0001530185286095631</v>
+        <v>0.004131215711950811</v>
       </c>
       <c r="X1">
-        <v>0.00415337319317881</v>
+        <v>0.0441170780966807</v>
       </c>
       <c r="Y1">
-        <v>0.006812599091287491</v>
+        <v>0.02830881558249385</v>
       </c>
       <c r="Z1">
-        <v>0.0001402202031142261</v>
+        <v>0.002792351658675057</v>
       </c>
       <c r="AA1">
-        <v>0.006812599091287491</v>
+        <v>0.02830881558249385</v>
       </c>
       <c r="AB1">
-        <v>0.01080129330867494</v>
+        <v>0.03220320498910477</v>
       </c>
       <c r="AC1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AD1">
-        <v>0.01080129330867494</v>
+        <v>0.03220320498910477</v>
       </c>
       <c r="AE1">
-        <v>0.01080129330867494</v>
+        <v>0.03220320498910477</v>
       </c>
       <c r="AF1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AG1">
-        <v>0.01080129330867494</v>
+        <v>0.03220320498910477</v>
       </c>
       <c r="AH1">
-        <v>0.01080129330867494</v>
+        <v>0.03220320498910477</v>
       </c>
       <c r="AI1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AJ1">
-        <v>0.01080129330867494</v>
+        <v>0.03220320498910477</v>
       </c>
       <c r="AK1">
-        <v>0.0001648236055669436</v>
+        <v>0.01261590551217859</v>
       </c>
       <c r="AL1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AM1">
-        <v>0.0001648236055669436</v>
+        <v>0.01261590551217859</v>
       </c>
       <c r="AN1">
-        <v>0.0001648236055669436</v>
+        <v>0.01261590551217859</v>
       </c>
       <c r="AO1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AP1">
-        <v>0.0001648236055669436</v>
+        <v>0.01261590551217859</v>
       </c>
       <c r="AQ1">
-        <v>0.00415337319317881</v>
+        <v>0.0441170780966807</v>
       </c>
       <c r="AR1">
-        <v>0.0001530185286095631</v>
+        <v>0.004131215711950811</v>
       </c>
       <c r="AS1">
-        <v>0.00415337319317881</v>
+        <v>0.0441170780966807</v>
       </c>
       <c r="AT1">
-        <v>0.003204207242957014</v>
+        <v>0.02873142008626384</v>
       </c>
       <c r="AU1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AV1">
-        <v>0.003204207242957014</v>
+        <v>0.02873142008626384</v>
       </c>
       <c r="AW1">
-        <v>0.003204207242957014</v>
+        <v>0.02873142008626384</v>
       </c>
       <c r="AX1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AY1">
-        <v>0.003204207242957014</v>
+        <v>0.02873142008626384</v>
       </c>
       <c r="AZ1">
-        <v>0.0001648236055669436</v>
+        <v>0.01261590551217859</v>
       </c>
       <c r="BA1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="BB1">
-        <v>0.0001648236055669436</v>
+        <v>0.01261590551217859</v>
       </c>
       <c r="BC1">
-        <v>0.0001648236055669436</v>
+        <v>0.01261590551217859</v>
       </c>
       <c r="BD1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="BE1">
-        <v>0.0001648236055669436</v>
+        <v>0.01261590551217859</v>
       </c>
     </row>
     <row r="2" spans="1:57">
       <c r="A2">
-        <v>0.01329569268477082</v>
+        <v>0.01460592263094856</v>
       </c>
       <c r="B2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="C2">
-        <v>0.01329569268477082</v>
+        <v>0.01460592263094856</v>
       </c>
       <c r="D2">
-        <v>0.01329569268477082</v>
+        <v>0.01460592263094856</v>
       </c>
       <c r="E2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="F2">
-        <v>0.01329569268477082</v>
+        <v>0.01460592263094856</v>
       </c>
       <c r="G2">
-        <v>0.03547460314413775</v>
+        <v>0.007592901447036864</v>
       </c>
       <c r="H2">
-        <v>0.1469630793008418</v>
+        <v>0.2096035334963209</v>
       </c>
       <c r="I2">
-        <v>0.03547460314413775</v>
+        <v>0.007592901447036864</v>
       </c>
       <c r="J2">
-        <v>0.01256237976152273</v>
+        <v>0.008488640835259492</v>
       </c>
       <c r="K2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="L2">
-        <v>0.01256237976152273</v>
+        <v>0.008488640835259492</v>
       </c>
       <c r="M2">
-        <v>0.03547460314413775</v>
+        <v>0.007592901447036864</v>
       </c>
       <c r="N2">
-        <v>0.1469630793008418</v>
+        <v>0.2096035334963209</v>
       </c>
       <c r="O2">
-        <v>0.03547460314413775</v>
+        <v>0.007592901447036864</v>
       </c>
       <c r="P2">
-        <v>0.03547460314413775</v>
+        <v>0.007592901447036864</v>
       </c>
       <c r="Q2">
-        <v>0.1469630793008418</v>
+        <v>0.2096035334963209</v>
       </c>
       <c r="R2">
-        <v>0.03547460314413775</v>
+        <v>0.007592901447036864</v>
       </c>
       <c r="S2">
-        <v>0.03547460314413775</v>
+        <v>0.007592901447036864</v>
       </c>
       <c r="T2">
-        <v>0.1469630793008418</v>
+        <v>0.2096035334963209</v>
       </c>
       <c r="U2">
-        <v>0.03547460314413775</v>
+        <v>0.007592901447036864</v>
       </c>
       <c r="V2">
-        <v>0.03547460314413775</v>
+        <v>0.007592901447036864</v>
       </c>
       <c r="W2">
-        <v>0.1469630793008418</v>
+        <v>0.2096035334963209</v>
       </c>
       <c r="X2">
-        <v>0.03547460314413775</v>
+        <v>0.007592901447036864</v>
       </c>
       <c r="Y2">
-        <v>0.0139836561524329</v>
+        <v>0.007572945135287123</v>
       </c>
       <c r="Z2">
-        <v>0.09801359405126905</v>
+        <v>0.1397738968482551</v>
       </c>
       <c r="AA2">
-        <v>0.0139836561524329</v>
+        <v>0.007572945135287123</v>
       </c>
       <c r="AB2">
-        <v>0.01256237976152273</v>
+        <v>0.008488640835259492</v>
       </c>
       <c r="AC2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AD2">
-        <v>0.01256237976152273</v>
+        <v>0.008488640835259492</v>
       </c>
       <c r="AE2">
-        <v>0.01256237976152273</v>
+        <v>0.008488640835259492</v>
       </c>
       <c r="AF2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AG2">
-        <v>0.01256237976152273</v>
+        <v>0.008488640835259492</v>
       </c>
       <c r="AH2">
-        <v>0.01256237976152273</v>
+        <v>0.008488640835259492</v>
       </c>
       <c r="AI2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AJ2">
-        <v>0.01256237976152273</v>
+        <v>0.008488640835259492</v>
       </c>
       <c r="AK2">
-        <v>0.006080735438400828</v>
+        <v>0.00573157557946751</v>
       </c>
       <c r="AL2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AM2">
-        <v>0.006080735438400828</v>
+        <v>0.00573157557946751</v>
       </c>
       <c r="AN2">
-        <v>0.006080735438400828</v>
+        <v>0.00573157557946751</v>
       </c>
       <c r="AO2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AP2">
-        <v>0.006080735438400828</v>
+        <v>0.00573157557946751</v>
       </c>
       <c r="AQ2">
-        <v>0.03547460314413775</v>
+        <v>0.007592901447036864</v>
       </c>
       <c r="AR2">
-        <v>0.1469630793008418</v>
+        <v>0.2096035334963209</v>
       </c>
       <c r="AS2">
-        <v>0.03547460314413775</v>
+        <v>0.007592901447036864</v>
       </c>
       <c r="AT2">
-        <v>0.01231794212044003</v>
+        <v>0.006449546903363136</v>
       </c>
       <c r="AU2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AV2">
-        <v>0.01231794212044003</v>
+        <v>0.006449546903363136</v>
       </c>
       <c r="AW2">
-        <v>0.01231794212044003</v>
+        <v>0.006449546903363136</v>
       </c>
       <c r="AX2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AY2">
-        <v>0.01231794212044003</v>
+        <v>0.006449546903363136</v>
       </c>
       <c r="AZ2">
-        <v>0.006080735438400828</v>
+        <v>0.00573157557946751</v>
       </c>
       <c r="BA2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="BB2">
-        <v>0.006080735438400828</v>
+        <v>0.00573157557946751</v>
       </c>
       <c r="BC2">
-        <v>0.006080735438400828</v>
+        <v>0.00573157557946751</v>
       </c>
       <c r="BD2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="BE2">
-        <v>0.006080735438400828</v>
+        <v>0.00573157557946751</v>
       </c>
     </row>
     <row r="3" spans="1:57">
       <c r="A3">
-        <v>0.009016779748564735</v>
+        <v>0.008827677126120309</v>
       </c>
       <c r="B3">
-        <v>0.326107825493968</v>
+        <v>0.396075168941436</v>
       </c>
       <c r="C3">
-        <v>0.009016779748564735</v>
+        <v>0.008827677126120309</v>
       </c>
       <c r="D3">
-        <v>0.009016779748564735</v>
+        <v>0.008827677126120309</v>
       </c>
       <c r="E3">
-        <v>0.326107825493968</v>
+        <v>0.396075168941436</v>
       </c>
       <c r="F3">
-        <v>0.009016779748564735</v>
+        <v>0.008827677126120309</v>
       </c>
       <c r="G3">
-        <v>0.01506335219405633</v>
+        <v>0.009184016523502319</v>
       </c>
       <c r="H3">
-        <v>0.3317162293534002</v>
+        <v>0.3271452180252837</v>
       </c>
       <c r="I3">
-        <v>0.01506335219405633</v>
+        <v>0.009184016523502319</v>
       </c>
       <c r="J3">
-        <v>0.01306817444397589</v>
+        <v>0.006838682809351938</v>
       </c>
       <c r="K3">
-        <v>0.326107825493968</v>
+        <v>0.396075168941436</v>
       </c>
       <c r="L3">
-        <v>0.01306817444397589</v>
+        <v>0.006838682809351938</v>
       </c>
       <c r="M3">
-        <v>0.01506335219405633</v>
+        <v>0.009184016523502319</v>
       </c>
       <c r="N3">
-        <v>0.3317162293534002</v>
+        <v>0.3271452180252837</v>
       </c>
       <c r="O3">
-        <v>0.01506335219405633</v>
+        <v>0.009184016523502319</v>
       </c>
       <c r="P3">
-        <v>0.01506335219405633</v>
+        <v>0.009184016523502319</v>
       </c>
       <c r="Q3">
-        <v>0.3317162293534002</v>
+        <v>0.3271452180252837</v>
       </c>
       <c r="R3">
-        <v>0.01506335219405633</v>
+        <v>0.009184016523502319</v>
       </c>
       <c r="S3">
-        <v>0.01506335219405633</v>
+        <v>0.009184016523502319</v>
       </c>
       <c r="T3">
-        <v>0.3317162293534002</v>
+        <v>0.3271452180252837</v>
       </c>
       <c r="U3">
-        <v>0.01506335219405633</v>
+        <v>0.009184016523502319</v>
       </c>
       <c r="V3">
-        <v>0.01506335219405633</v>
+        <v>0.009184016523502319</v>
       </c>
       <c r="W3">
-        <v>0.3317162293534002</v>
+        <v>0.3271452180252837</v>
       </c>
       <c r="X3">
-        <v>0.01506335219405633</v>
+        <v>0.009184016523502319</v>
       </c>
       <c r="Y3">
-        <v>0.01229076004851318</v>
+        <v>0.006869978102312557</v>
       </c>
       <c r="Z3">
-        <v>0.3298467614002561</v>
+        <v>0.3501218683306678</v>
       </c>
       <c r="AA3">
-        <v>0.01229076004851318</v>
+        <v>0.006869978102312557</v>
       </c>
       <c r="AB3">
-        <v>0.01306817444397589</v>
+        <v>0.006838682809351938</v>
       </c>
       <c r="AC3">
-        <v>0.326107825493968</v>
+        <v>0.396075168941436</v>
       </c>
       <c r="AD3">
-        <v>0.01306817444397589</v>
+        <v>0.006838682809351938</v>
       </c>
       <c r="AE3">
-        <v>0.01306817444397589</v>
+        <v>0.006838682809351938</v>
       </c>
       <c r="AF3">
-        <v>0.326107825493968</v>
+        <v>0.396075168941436</v>
       </c>
       <c r="AG3">
-        <v>0.01306817444397589</v>
+        <v>0.006838682809351938</v>
       </c>
       <c r="AH3">
-        <v>0.01306817444397589</v>
+        <v>0.006838682809351938</v>
       </c>
       <c r="AI3">
-        <v>0.326107825493968</v>
+        <v>0.396075168941436</v>
       </c>
       <c r="AJ3">
-        <v>0.01306817444397589</v>
+        <v>0.006838682809351938</v>
       </c>
       <c r="AK3">
-        <v>0.009349635184816175</v>
+        <v>0.005775549477638912</v>
       </c>
       <c r="AL3">
-        <v>0.326107825493968</v>
+        <v>0.396075168941436</v>
       </c>
       <c r="AM3">
-        <v>0.009349635184816175</v>
+        <v>0.005775549477638912</v>
       </c>
       <c r="AN3">
-        <v>0.009349635184816175</v>
+        <v>0.005775549477638912</v>
       </c>
       <c r="AO3">
-        <v>0.326107825493968</v>
+        <v>0.396075168941436</v>
       </c>
       <c r="AP3">
-        <v>0.009349635184816175</v>
+        <v>0.005775549477638912</v>
       </c>
       <c r="AQ3">
-        <v>0.01506335219405633</v>
+        <v>0.009184016523502319</v>
       </c>
       <c r="AR3">
-        <v>0.3317162293534002</v>
+        <v>0.3271452180252837</v>
       </c>
       <c r="AS3">
-        <v>0.01506335219405633</v>
+        <v>0.009184016523502319</v>
       </c>
       <c r="AT3">
-        <v>0.01441863934244628</v>
+        <v>0.006175684703762482</v>
       </c>
       <c r="AU3">
-        <v>0.326107825493968</v>
+        <v>0.396075168941436</v>
       </c>
       <c r="AV3">
-        <v>0.01441863934244628</v>
+        <v>0.006175684703762482</v>
       </c>
       <c r="AW3">
-        <v>0.01441863934244628</v>
+        <v>0.006175684703762482</v>
       </c>
       <c r="AX3">
-        <v>0.326107825493968</v>
+        <v>0.396075168941436</v>
       </c>
       <c r="AY3">
-        <v>0.01441863934244628</v>
+        <v>0.006175684703762482</v>
       </c>
       <c r="AZ3">
-        <v>0.009349635184816175</v>
+        <v>0.005775549477638912</v>
       </c>
       <c r="BA3">
-        <v>0.326107825493968</v>
+        <v>0.396075168941436</v>
       </c>
       <c r="BB3">
-        <v>0.009349635184816175</v>
+        <v>0.005775549477638912</v>
       </c>
       <c r="BC3">
-        <v>0.009349635184816175</v>
+        <v>0.005775549477638912</v>
       </c>
       <c r="BD3">
-        <v>0.326107825493968</v>
+        <v>0.396075168941436</v>
       </c>
       <c r="BE3">
-        <v>0.009349635184816175</v>
+        <v>0.005775549477638912</v>
       </c>
     </row>
     <row r="4" spans="1:57">
       <c r="A4">
-        <v>0.01080975467967811</v>
+        <v>0.01189379243929846</v>
       </c>
       <c r="B4">
-        <v>0.2171924988317014</v>
+        <v>0.1430970420835792</v>
       </c>
       <c r="C4">
-        <v>0.01080975467967811</v>
+        <v>0.01189379243929846</v>
       </c>
       <c r="D4">
-        <v>0.01080975467967811</v>
+        <v>0.01189379243929846</v>
       </c>
       <c r="E4">
-        <v>0.2171924988317014</v>
+        <v>0.1430970420835792</v>
       </c>
       <c r="F4">
-        <v>0.01080975467967811</v>
+        <v>0.01189379243929846</v>
       </c>
       <c r="G4">
-        <v>0.01669895148551608</v>
+        <v>0.006172366134497694</v>
       </c>
       <c r="H4">
-        <v>0.1769669385797322</v>
+        <v>0.1426807817772778</v>
       </c>
       <c r="I4">
-        <v>0.01669895148551608</v>
+        <v>0.006172366134497694</v>
       </c>
       <c r="J4">
-        <v>0.01003982395500032</v>
+        <v>0.005667464598099573</v>
       </c>
       <c r="K4">
-        <v>0.2171924988317014</v>
+        <v>0.1430970420835792</v>
       </c>
       <c r="L4">
-        <v>0.01003982395500032</v>
+        <v>0.005667464598099573</v>
       </c>
       <c r="M4">
-        <v>0.01669895148551608</v>
+        <v>0.006172366134497694</v>
       </c>
       <c r="N4">
-        <v>0.1769669385797322</v>
+        <v>0.1426807817772778</v>
       </c>
       <c r="O4">
-        <v>0.01669895148551608</v>
+        <v>0.006172366134497694</v>
       </c>
       <c r="P4">
-        <v>0.01669895148551608</v>
+        <v>0.006172366134497694</v>
       </c>
       <c r="Q4">
-        <v>0.1769669385797322</v>
+        <v>0.1426807817772778</v>
       </c>
       <c r="R4">
-        <v>0.01669895148551608</v>
+        <v>0.006172366134497694</v>
       </c>
       <c r="S4">
-        <v>0.01669895148551608</v>
+        <v>0.006172366134497694</v>
       </c>
       <c r="T4">
-        <v>0.1769669385797322</v>
+        <v>0.1426807817772778</v>
       </c>
       <c r="U4">
-        <v>0.01669895148551608</v>
+        <v>0.006172366134497694</v>
       </c>
       <c r="V4">
-        <v>0.01669895148551608</v>
+        <v>0.006172366134497694</v>
       </c>
       <c r="W4">
-        <v>0.1769669385797322</v>
+        <v>0.1426807817772778</v>
       </c>
       <c r="X4">
-        <v>0.01669895148551608</v>
+        <v>0.006172366134497694</v>
       </c>
       <c r="Y4">
-        <v>0.01031864210849662</v>
+        <v>0.004890176770189002</v>
       </c>
       <c r="Z4">
-        <v>0.1903754586637219</v>
+        <v>0.1428195352127116</v>
       </c>
       <c r="AA4">
-        <v>0.01031864210849662</v>
+        <v>0.004890176770189002</v>
       </c>
       <c r="AB4">
-        <v>0.01003982395500032</v>
+        <v>0.005667464598099573</v>
       </c>
       <c r="AC4">
-        <v>0.2171924988317014</v>
+        <v>0.1430970420835792</v>
       </c>
       <c r="AD4">
-        <v>0.01003982395500032</v>
+        <v>0.005667464598099573</v>
       </c>
       <c r="AE4">
-        <v>0.01003982395500032</v>
+        <v>0.005667464598099573</v>
       </c>
       <c r="AF4">
-        <v>0.2171924988317014</v>
+        <v>0.1430970420835792</v>
       </c>
       <c r="AG4">
-        <v>0.01003982395500032</v>
+        <v>0.005667464598099573</v>
       </c>
       <c r="AH4">
-        <v>0.01003982395500032</v>
+        <v>0.005667464598099573</v>
       </c>
       <c r="AI4">
-        <v>0.2171924988317014</v>
+        <v>0.1430970420835792</v>
       </c>
       <c r="AJ4">
-        <v>0.01003982395500032</v>
+        <v>0.005667464598099573</v>
       </c>
       <c r="AK4">
-        <v>0.0076861237269795</v>
+        <v>0.002694506432213508</v>
       </c>
       <c r="AL4">
-        <v>0.2171924988317014</v>
+        <v>0.1430970420835792</v>
       </c>
       <c r="AM4">
-        <v>0.0076861237269795</v>
+        <v>0.002694506432213508</v>
       </c>
       <c r="AN4">
-        <v>0.0076861237269795</v>
+        <v>0.002694506432213508</v>
       </c>
       <c r="AO4">
-        <v>0.2171924988317014</v>
+        <v>0.1430970420835792</v>
       </c>
       <c r="AP4">
-        <v>0.0076861237269795</v>
+        <v>0.002694506432213508</v>
       </c>
       <c r="AQ4">
-        <v>0.01669895148551608</v>
+        <v>0.006172366134497694</v>
       </c>
       <c r="AR4">
-        <v>0.1769669385797322</v>
+        <v>0.1426807817772778</v>
       </c>
       <c r="AS4">
-        <v>0.01669895148551608</v>
+        <v>0.006172366134497694</v>
       </c>
       <c r="AT4">
-        <v>0.009783180380107722</v>
+        <v>0.003592021984366611</v>
       </c>
       <c r="AU4">
-        <v>0.2171924988317014</v>
+        <v>0.1430970420835792</v>
       </c>
       <c r="AV4">
-        <v>0.009783180380107722</v>
+        <v>0.003592021984366611</v>
       </c>
       <c r="AW4">
-        <v>0.009783180380107722</v>
+        <v>0.003592021984366611</v>
       </c>
       <c r="AX4">
-        <v>0.2171924988317014</v>
+        <v>0.1430970420835792</v>
       </c>
       <c r="AY4">
-        <v>0.009783180380107722</v>
+        <v>0.003592021984366611</v>
       </c>
       <c r="AZ4">
-        <v>0.0076861237269795</v>
+        <v>0.002694506432213508</v>
       </c>
       <c r="BA4">
-        <v>0.2171924988317014</v>
+        <v>0.1430970420835792</v>
       </c>
       <c r="BB4">
-        <v>0.0076861237269795</v>
+        <v>0.002694506432213508</v>
       </c>
       <c r="BC4">
-        <v>0.0076861237269795</v>
+        <v>0.002694506432213508</v>
       </c>
       <c r="BD4">
-        <v>0.2171924988317014</v>
+        <v>0.1430970420835792</v>
       </c>
       <c r="BE4">
-        <v>0.0076861237269795</v>
+        <v>0.002694506432213508</v>
       </c>
     </row>
     <row r="5" spans="1:57">
       <c r="A5">
-        <v>0.01089133042749333</v>
+        <v>0.007020063450574888</v>
       </c>
       <c r="B5">
-        <v>0.1466277815139906</v>
+        <v>0.1448482868644593</v>
       </c>
       <c r="C5">
-        <v>0.01089133042749333</v>
+        <v>0.007020063450574888</v>
       </c>
       <c r="D5">
-        <v>0.01089133042749333</v>
+        <v>0.007020063450574888</v>
       </c>
       <c r="E5">
-        <v>0.1466277815139906</v>
+        <v>0.1448482868644593</v>
       </c>
       <c r="F5">
-        <v>0.01089133042749333</v>
+        <v>0.007020063450574888</v>
       </c>
       <c r="G5">
-        <v>0.001845113746186173</v>
+        <v>0.009108166267423327</v>
       </c>
       <c r="H5">
-        <v>0.1350304976632463</v>
+        <v>0.1318822494666863</v>
       </c>
       <c r="I5">
-        <v>0.001845113746186173</v>
+        <v>0.009108166267423327</v>
       </c>
       <c r="J5">
-        <v>0.009512934771852246</v>
+        <v>0.004908398109682398</v>
       </c>
       <c r="K5">
-        <v>0.1466277815139906</v>
+        <v>0.1448482868644593</v>
       </c>
       <c r="L5">
-        <v>0.009512934771852246</v>
+        <v>0.004908398109682398</v>
       </c>
       <c r="M5">
-        <v>0.001845113746186173</v>
+        <v>0.009108166267423327</v>
       </c>
       <c r="N5">
-        <v>0.1350304976632463</v>
+        <v>0.1318822494666863</v>
       </c>
       <c r="O5">
-        <v>0.001845113746186173</v>
+        <v>0.009108166267423327</v>
       </c>
       <c r="P5">
-        <v>0.001845113746186173</v>
+        <v>0.009108166267423327</v>
       </c>
       <c r="Q5">
-        <v>0.1350304976632463</v>
+        <v>0.1318822494666863</v>
       </c>
       <c r="R5">
-        <v>0.001845113746186173</v>
+        <v>0.009108166267423327</v>
       </c>
       <c r="S5">
-        <v>0.001845113746186173</v>
+        <v>0.009108166267423327</v>
       </c>
       <c r="T5">
-        <v>0.1350304976632463</v>
+        <v>0.1318822494666863</v>
       </c>
       <c r="U5">
-        <v>0.001845113746186173</v>
+        <v>0.009108166267423327</v>
       </c>
       <c r="V5">
-        <v>0.001845113746186173</v>
+        <v>0.009108166267423327</v>
       </c>
       <c r="W5">
-        <v>0.1350304976632463</v>
+        <v>0.1318822494666863</v>
       </c>
       <c r="X5">
-        <v>0.001845113746186173</v>
+        <v>0.009108166267423327</v>
       </c>
       <c r="Y5">
-        <v>0.007562330893504463</v>
+        <v>0.005102479196887717</v>
       </c>
       <c r="Z5">
-        <v>0.1388962589468278</v>
+        <v>0.1362042619326106</v>
       </c>
       <c r="AA5">
-        <v>0.007562330893504463</v>
+        <v>0.005102479196887717</v>
       </c>
       <c r="AB5">
-        <v>0.009512934771852246</v>
+        <v>0.004908398109682398</v>
       </c>
       <c r="AC5">
-        <v>0.1466277815139906</v>
+        <v>0.1448482868644593</v>
       </c>
       <c r="AD5">
-        <v>0.009512934771852246</v>
+        <v>0.004908398109682398</v>
       </c>
       <c r="AE5">
-        <v>0.009512934771852246</v>
+        <v>0.004908398109682398</v>
       </c>
       <c r="AF5">
-        <v>0.1466277815139906</v>
+        <v>0.1448482868644593</v>
       </c>
       <c r="AG5">
-        <v>0.009512934771852246</v>
+        <v>0.004908398109682398</v>
       </c>
       <c r="AH5">
-        <v>0.009512934771852246</v>
+        <v>0.004908398109682398</v>
       </c>
       <c r="AI5">
-        <v>0.1466277815139906</v>
+        <v>0.1448482868644593</v>
       </c>
       <c r="AJ5">
-        <v>0.009512934771852246</v>
+        <v>0.004908398109682398</v>
       </c>
       <c r="AK5">
-        <v>0.006519731710468045</v>
+        <v>0.003487797836030551</v>
       </c>
       <c r="AL5">
-        <v>0.1466277815139906</v>
+        <v>0.1448482868644593</v>
       </c>
       <c r="AM5">
-        <v>0.006519731710468045</v>
+        <v>0.003487797836030551</v>
       </c>
       <c r="AN5">
-        <v>0.006519731710468045</v>
+        <v>0.003487797836030551</v>
       </c>
       <c r="AO5">
-        <v>0.1466277815139906</v>
+        <v>0.1448482868644593</v>
       </c>
       <c r="AP5">
-        <v>0.006519731710468045</v>
+        <v>0.003487797836030551</v>
       </c>
       <c r="AQ5">
-        <v>0.001845113746186173</v>
+        <v>0.009108166267423327</v>
       </c>
       <c r="AR5">
-        <v>0.1350304976632463</v>
+        <v>0.1318822494666863</v>
       </c>
       <c r="AS5">
-        <v>0.001845113746186173</v>
+        <v>0.009108166267423327</v>
       </c>
       <c r="AT5">
-        <v>0.009053469553305216</v>
+        <v>0.004204509662718235</v>
       </c>
       <c r="AU5">
-        <v>0.1466277815139906</v>
+        <v>0.1448482868644593</v>
       </c>
       <c r="AV5">
-        <v>0.009053469553305216</v>
+        <v>0.004204509662718235</v>
       </c>
       <c r="AW5">
-        <v>0.009053469553305216</v>
+        <v>0.004204509662718235</v>
       </c>
       <c r="AX5">
-        <v>0.1466277815139906</v>
+        <v>0.1448482868644593</v>
       </c>
       <c r="AY5">
-        <v>0.009053469553305216</v>
+        <v>0.004204509662718235</v>
       </c>
       <c r="AZ5">
-        <v>0.006519731710468045</v>
+        <v>0.003487797836030551</v>
       </c>
       <c r="BA5">
-        <v>0.1466277815139906</v>
+        <v>0.1448482868644593</v>
       </c>
       <c r="BB5">
-        <v>0.006519731710468045</v>
+        <v>0.003487797836030551</v>
       </c>
       <c r="BC5">
-        <v>0.006519731710468045</v>
+        <v>0.003487797836030551</v>
       </c>
       <c r="BD5">
-        <v>0.1466277815139906</v>
+        <v>0.1448482868644593</v>
       </c>
       <c r="BE5">
-        <v>0.006519731710468045</v>
+        <v>0.003487797836030551</v>
       </c>
     </row>
     <row r="6" spans="1:57">
       <c r="A6">
-        <v>0.007484115743621659</v>
+        <v>0.006105371091459948</v>
       </c>
       <c r="B6">
-        <v>0.1228699079585041</v>
+        <v>0.08568051951151724</v>
       </c>
       <c r="C6">
-        <v>0.007484115743621659</v>
+        <v>0.006105371091459948</v>
       </c>
       <c r="D6">
-        <v>0.007484115743621659</v>
+        <v>0.006105371091459948</v>
       </c>
       <c r="E6">
-        <v>0.1228699079585041</v>
+        <v>0.08568051951151724</v>
       </c>
       <c r="F6">
-        <v>0.007484115743621659</v>
+        <v>0.006105371091459948</v>
       </c>
       <c r="G6">
-        <v>0.0001849315068493151</v>
+        <v>0.006328575760998325</v>
       </c>
       <c r="H6">
-        <v>0.1469265467189451</v>
+        <v>0.1327550294386663</v>
       </c>
       <c r="I6">
-        <v>0.0001849315068493151</v>
+        <v>0.006328575760998325</v>
       </c>
       <c r="J6">
-        <v>0.008351383692089775</v>
+        <v>0.004707971756326143</v>
       </c>
       <c r="K6">
-        <v>0.1228699079585041</v>
+        <v>0.08568051951151724</v>
       </c>
       <c r="L6">
-        <v>0.008351383692089775</v>
+        <v>0.004707971756326143</v>
       </c>
       <c r="M6">
-        <v>0.0001849315068493151</v>
+        <v>0.006328575760998325</v>
       </c>
       <c r="N6">
-        <v>0.1469265467189451</v>
+        <v>0.1327550294386663</v>
       </c>
       <c r="O6">
-        <v>0.0001849315068493151</v>
+        <v>0.006328575760998325</v>
       </c>
       <c r="P6">
-        <v>0.0001849315068493151</v>
+        <v>0.006328575760998325</v>
       </c>
       <c r="Q6">
-        <v>0.1469265467189451</v>
+        <v>0.1327550294386663</v>
       </c>
       <c r="R6">
-        <v>0.0001849315068493151</v>
+        <v>0.006328575760998325</v>
       </c>
       <c r="S6">
-        <v>0.0001849315068493151</v>
+        <v>0.006328575760998325</v>
       </c>
       <c r="T6">
-        <v>0.1469265467189451</v>
+        <v>0.1327550294386663</v>
       </c>
       <c r="U6">
-        <v>0.0001849315068493151</v>
+        <v>0.006328575760998325</v>
       </c>
       <c r="V6">
-        <v>0.0001849315068493151</v>
+        <v>0.006328575760998325</v>
       </c>
       <c r="W6">
-        <v>0.1469265467189451</v>
+        <v>0.1327550294386663</v>
       </c>
       <c r="X6">
-        <v>0.0001849315068493151</v>
+        <v>0.006328575760998325</v>
       </c>
       <c r="Y6">
-        <v>0.006571276703108419</v>
+        <v>0.00446100092028795</v>
       </c>
       <c r="Z6">
-        <v>0.1389076671321314</v>
+        <v>0.1170635261296166</v>
       </c>
       <c r="AA6">
-        <v>0.006571276703108419</v>
+        <v>0.00446100092028795</v>
       </c>
       <c r="AB6">
-        <v>0.008351383692089775</v>
+        <v>0.004707971756326143</v>
       </c>
       <c r="AC6">
-        <v>0.1228699079585041</v>
+        <v>0.08568051951151724</v>
       </c>
       <c r="AD6">
-        <v>0.008351383692089775</v>
+        <v>0.004707971756326143</v>
       </c>
       <c r="AE6">
-        <v>0.008351383692089775</v>
+        <v>0.004707971756326143</v>
       </c>
       <c r="AF6">
-        <v>0.1228699079585041</v>
+        <v>0.08568051951151724</v>
       </c>
       <c r="AG6">
-        <v>0.008351383692089775</v>
+        <v>0.004707971756326143</v>
       </c>
       <c r="AH6">
-        <v>0.008351383692089775</v>
+        <v>0.004707971756326143</v>
       </c>
       <c r="AI6">
-        <v>0.1228699079585041</v>
+        <v>0.08568051951151724</v>
       </c>
       <c r="AJ6">
-        <v>0.008351383692089775</v>
+        <v>0.004707971756326143</v>
       </c>
       <c r="AK6">
-        <v>0.006204235323275257</v>
+        <v>0.003033271827856376</v>
       </c>
       <c r="AL6">
-        <v>0.1228699079585041</v>
+        <v>0.08568051951151724</v>
       </c>
       <c r="AM6">
-        <v>0.006204235323275257</v>
+        <v>0.003033271827856376</v>
       </c>
       <c r="AN6">
-        <v>0.006204235323275257</v>
+        <v>0.003033271827856376</v>
       </c>
       <c r="AO6">
-        <v>0.1228699079585041</v>
+        <v>0.08568051951151724</v>
       </c>
       <c r="AP6">
-        <v>0.006204235323275257</v>
+        <v>0.003033271827856376</v>
       </c>
       <c r="AQ6">
-        <v>0.0001849315068493151</v>
+        <v>0.006328575760998325</v>
       </c>
       <c r="AR6">
-        <v>0.1469265467189451</v>
+        <v>0.1327550294386663</v>
       </c>
       <c r="AS6">
-        <v>0.0001849315068493151</v>
+        <v>0.006328575760998325</v>
       </c>
       <c r="AT6">
-        <v>0.008640473008245815</v>
+        <v>0.004242171977948208</v>
       </c>
       <c r="AU6">
-        <v>0.1228699079585041</v>
+        <v>0.08568051951151724</v>
       </c>
       <c r="AV6">
-        <v>0.008640473008245815</v>
+        <v>0.004242171977948208</v>
       </c>
       <c r="AW6">
-        <v>0.008640473008245815</v>
+        <v>0.004242171977948208</v>
       </c>
       <c r="AX6">
-        <v>0.1228699079585041</v>
+        <v>0.08568051951151724</v>
       </c>
       <c r="AY6">
-        <v>0.008640473008245815</v>
+        <v>0.004242171977948208</v>
       </c>
       <c r="AZ6">
-        <v>0.006204235323275257</v>
+        <v>0.003033271827856376</v>
       </c>
       <c r="BA6">
-        <v>0.1228699079585041</v>
+        <v>0.08568051951151724</v>
       </c>
       <c r="BB6">
-        <v>0.006204235323275257</v>
+        <v>0.003033271827856376</v>
       </c>
       <c r="BC6">
-        <v>0.006204235323275257</v>
+        <v>0.003033271827856376</v>
       </c>
       <c r="BD6">
-        <v>0.1228699079585041</v>
+        <v>0.08568051951151724</v>
       </c>
       <c r="BE6">
-        <v>0.006204235323275257</v>
+        <v>0.003033271827856376</v>
       </c>
     </row>
     <row r="7" spans="1:57">
       <c r="A7">
-        <v>0.005554174131977045</v>
+        <v>0.007792132306019362</v>
       </c>
       <c r="B7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="C7">
-        <v>0.005554174131977045</v>
+        <v>0.007792132306019362</v>
       </c>
       <c r="D7">
-        <v>0.005554174131977045</v>
+        <v>0.007792132306019362</v>
       </c>
       <c r="E7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="F7">
-        <v>0.005554174131977045</v>
+        <v>0.007792132306019362</v>
       </c>
       <c r="G7">
-        <v>0.0001849315068493151</v>
+        <v>0.005366987015587355</v>
       </c>
       <c r="H7">
-        <v>0.03976329111914859</v>
+        <v>0.03735581464316458</v>
       </c>
       <c r="I7">
-        <v>0.0001849315068493151</v>
+        <v>0.005366987015587355</v>
       </c>
       <c r="J7">
-        <v>0.00531149095487475</v>
+        <v>0.004642694803025653</v>
       </c>
       <c r="K7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="L7">
-        <v>0.00531149095487475</v>
+        <v>0.004642694803025653</v>
       </c>
       <c r="M7">
-        <v>0.0001849315068493151</v>
+        <v>0.005366987015587355</v>
       </c>
       <c r="N7">
-        <v>0.03976329111914859</v>
+        <v>0.03735581464316458</v>
       </c>
       <c r="O7">
-        <v>0.0001849315068493151</v>
+        <v>0.005366987015587355</v>
       </c>
       <c r="P7">
-        <v>0.0001849315068493151</v>
+        <v>0.005366987015587355</v>
       </c>
       <c r="Q7">
-        <v>0.03976329111914859</v>
+        <v>0.03735581464316458</v>
       </c>
       <c r="R7">
-        <v>0.0001849315068493151</v>
+        <v>0.005366987015587355</v>
       </c>
       <c r="S7">
-        <v>0.0001849315068493151</v>
+        <v>0.005366987015587355</v>
       </c>
       <c r="T7">
-        <v>0.03976329111914859</v>
+        <v>0.03735581464316458</v>
       </c>
       <c r="U7">
-        <v>0.0001849315068493151</v>
+        <v>0.005366987015587355</v>
       </c>
       <c r="V7">
-        <v>0.0001849315068493151</v>
+        <v>0.005366987015587355</v>
       </c>
       <c r="W7">
-        <v>0.03976329111914859</v>
+        <v>0.03735581464316458</v>
       </c>
       <c r="X7">
-        <v>0.0001849315068493151</v>
+        <v>0.005366987015587355</v>
       </c>
       <c r="Y7">
-        <v>0.003855230184347192</v>
+        <v>0.004156788821189753</v>
       </c>
       <c r="Z7">
-        <v>0.02654706859680691</v>
+        <v>0.02494208427948423</v>
       </c>
       <c r="AA7">
-        <v>0.003855230184347192</v>
+        <v>0.004156788821189753</v>
       </c>
       <c r="AB7">
-        <v>0.00531149095487475</v>
+        <v>0.004642694803025653</v>
       </c>
       <c r="AC7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AD7">
-        <v>0.00531149095487475</v>
+        <v>0.004642694803025653</v>
       </c>
       <c r="AE7">
-        <v>0.00531149095487475</v>
+        <v>0.004642694803025653</v>
       </c>
       <c r="AF7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AG7">
-        <v>0.00531149095487475</v>
+        <v>0.004642694803025653</v>
       </c>
       <c r="AH7">
-        <v>0.00531149095487475</v>
+        <v>0.004642694803025653</v>
       </c>
       <c r="AI7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AJ7">
-        <v>0.00531149095487475</v>
+        <v>0.004642694803025653</v>
       </c>
       <c r="AK7">
-        <v>0.002777857982041016</v>
+        <v>0.002579877760319154</v>
       </c>
       <c r="AL7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AM7">
-        <v>0.002777857982041016</v>
+        <v>0.002579877760319154</v>
       </c>
       <c r="AN7">
-        <v>0.002777857982041016</v>
+        <v>0.002579877760319154</v>
       </c>
       <c r="AO7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AP7">
-        <v>0.002777857982041016</v>
+        <v>0.002579877760319154</v>
       </c>
       <c r="AQ7">
-        <v>0.0001849315068493151</v>
+        <v>0.005366987015587355</v>
       </c>
       <c r="AR7">
-        <v>0.03976329111914859</v>
+        <v>0.03735581464316458</v>
       </c>
       <c r="AS7">
-        <v>0.0001849315068493151</v>
+        <v>0.005366987015587355</v>
       </c>
       <c r="AT7">
-        <v>0.005230596562507317</v>
+        <v>0.003592882302027751</v>
       </c>
       <c r="AU7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AV7">
-        <v>0.005230596562507317</v>
+        <v>0.003592882302027751</v>
       </c>
       <c r="AW7">
-        <v>0.005230596562507317</v>
+        <v>0.003592882302027751</v>
       </c>
       <c r="AX7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AY7">
-        <v>0.005230596562507317</v>
+        <v>0.003592882302027751</v>
       </c>
       <c r="AZ7">
-        <v>0.002777857982041016</v>
+        <v>0.002579877760319154</v>
       </c>
       <c r="BA7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="BB7">
-        <v>0.002777857982041016</v>
+        <v>0.002579877760319154</v>
       </c>
       <c r="BC7">
-        <v>0.002777857982041016</v>
+        <v>0.002579877760319154</v>
       </c>
       <c r="BD7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="BE7">
-        <v>0.002777857982041016</v>
+        <v>0.002579877760319154</v>
       </c>
     </row>
     <row r="8" spans="1:57">
       <c r="A8">
-        <v>0.0007570548562017816</v>
+        <v>0.004276090778868289</v>
       </c>
       <c r="B8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="C8">
-        <v>0.0007570548562017816</v>
+        <v>0.004276090778868289</v>
       </c>
       <c r="D8">
-        <v>0.0007570548562017816</v>
+        <v>0.004276090778868289</v>
       </c>
       <c r="E8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="F8">
-        <v>0.0007570548562017816</v>
+        <v>0.004276090778868289</v>
       </c>
       <c r="G8">
-        <v>0.0001849315068493151</v>
+        <v>0.002197409566330036</v>
       </c>
       <c r="H8">
-        <v>0.02217436167885712</v>
+        <v>0.0141237196614283</v>
       </c>
       <c r="I8">
-        <v>0.0001849315068493151</v>
+        <v>0.002197409566330036</v>
       </c>
       <c r="J8">
-        <v>0.001256368340240204</v>
+        <v>0.002503492017771478</v>
       </c>
       <c r="K8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="L8">
-        <v>0.001256368340240204</v>
+        <v>0.002503492017771478</v>
       </c>
       <c r="M8">
-        <v>0.0001849315068493151</v>
+        <v>0.002197409566330036</v>
       </c>
       <c r="N8">
-        <v>0.02217436167885712</v>
+        <v>0.0141237196614283</v>
       </c>
       <c r="O8">
-        <v>0.0001849315068493151</v>
+        <v>0.002197409566330036</v>
       </c>
       <c r="P8">
-        <v>0.0001849315068493151</v>
+        <v>0.002197409566330036</v>
       </c>
       <c r="Q8">
-        <v>0.02217436167885712</v>
+        <v>0.0141237196614283</v>
       </c>
       <c r="R8">
-        <v>0.0001849315068493151</v>
+        <v>0.002197409566330036</v>
       </c>
       <c r="S8">
-        <v>0.0001849315068493151</v>
+        <v>0.002197409566330036</v>
       </c>
       <c r="T8">
-        <v>0.02217436167885712</v>
+        <v>0.0141237196614283</v>
       </c>
       <c r="U8">
-        <v>0.0001849315068493151</v>
+        <v>0.002197409566330036</v>
       </c>
       <c r="V8">
-        <v>0.0001849315068493151</v>
+        <v>0.002197409566330036</v>
       </c>
       <c r="W8">
-        <v>0.02217436167885712</v>
+        <v>0.0141237196614283</v>
       </c>
       <c r="X8">
-        <v>0.0001849315068493151</v>
+        <v>0.002197409566330036</v>
       </c>
       <c r="Y8">
-        <v>0.0007914360112777169</v>
+        <v>0.002350507755886142</v>
       </c>
       <c r="Z8">
-        <v>0.0148211156366126</v>
+        <v>0.009454020958326719</v>
       </c>
       <c r="AA8">
-        <v>0.0007914360112777169</v>
+        <v>0.002350507755886142</v>
       </c>
       <c r="AB8">
-        <v>0.001256368340240204</v>
+        <v>0.002503492017771478</v>
       </c>
       <c r="AC8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AD8">
-        <v>0.001256368340240204</v>
+        <v>0.002503492017771478</v>
       </c>
       <c r="AE8">
-        <v>0.001256368340240204</v>
+        <v>0.002503492017771478</v>
       </c>
       <c r="AF8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AG8">
-        <v>0.001256368340240204</v>
+        <v>0.002503492017771478</v>
       </c>
       <c r="AH8">
-        <v>0.001256368340240204</v>
+        <v>0.002503492017771478</v>
       </c>
       <c r="AI8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AJ8">
-        <v>0.001256368340240204</v>
+        <v>0.002503492017771478</v>
       </c>
       <c r="AK8">
-        <v>0.0001648236055669436</v>
+        <v>0.002121088326893522</v>
       </c>
       <c r="AL8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AM8">
-        <v>0.0001648236055669436</v>
+        <v>0.002121088326893522</v>
       </c>
       <c r="AN8">
-        <v>0.0001648236055669436</v>
+        <v>0.002121088326893522</v>
       </c>
       <c r="AO8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AP8">
-        <v>0.0001648236055669436</v>
+        <v>0.002121088326893522</v>
       </c>
       <c r="AQ8">
-        <v>0.0001849315068493151</v>
+        <v>0.002197409566330036</v>
       </c>
       <c r="AR8">
-        <v>0.02217436167885712</v>
+        <v>0.0141237196614283</v>
       </c>
       <c r="AS8">
-        <v>0.0001849315068493151</v>
+        <v>0.002197409566330036</v>
       </c>
       <c r="AT8">
-        <v>0.001422806168253012</v>
+        <v>0.001912625764072542</v>
       </c>
       <c r="AU8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AV8">
-        <v>0.001422806168253012</v>
+        <v>0.001912625764072542</v>
       </c>
       <c r="AW8">
-        <v>0.001422806168253012</v>
+        <v>0.001912625764072542</v>
       </c>
       <c r="AX8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AY8">
-        <v>0.001422806168253012</v>
+        <v>0.001912625764072542</v>
       </c>
       <c r="AZ8">
-        <v>0.0001648236055669436</v>
+        <v>0.002121088326893522</v>
       </c>
       <c r="BA8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="BB8">
-        <v>0.0001648236055669436</v>
+        <v>0.002121088326893522</v>
       </c>
       <c r="BC8">
-        <v>0.0001648236055669436</v>
+        <v>0.002121088326893522</v>
       </c>
       <c r="BD8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="BE8">
-        <v>0.0001648236055669436</v>
+        <v>0.002121088326893522</v>
       </c>
     </row>
     <row r="9" spans="1:57">
       <c r="A9">
-        <v>0.000235106866757617</v>
+        <v>0.001677694408127644</v>
       </c>
       <c r="B9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="C9">
-        <v>0.000235106866757617</v>
+        <v>0.001677694408127644</v>
       </c>
       <c r="D9">
-        <v>0.000235106866757617</v>
+        <v>0.001677694408127644</v>
       </c>
       <c r="E9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="F9">
-        <v>0.000235106866757617</v>
+        <v>0.001677694408127644</v>
       </c>
       <c r="G9">
-        <v>0.0001849315068493151</v>
+        <v>0.001707954726293864</v>
       </c>
       <c r="H9">
-        <v>0.0001530185286095631</v>
+        <v>0.0001612188896106683</v>
       </c>
       <c r="I9">
-        <v>0.0001849315068493151</v>
+        <v>0.001707954726293864</v>
       </c>
       <c r="J9">
-        <v>0.0002451613829154453</v>
+        <v>0.001293297022188149</v>
       </c>
       <c r="K9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="L9">
-        <v>0.0002451613829154453</v>
+        <v>0.001293297022188149</v>
       </c>
       <c r="M9">
-        <v>0.0001849315068493151</v>
+        <v>0.001707954726293864</v>
       </c>
       <c r="N9">
-        <v>0.0001530185286095631</v>
+        <v>0.0001612188896106683</v>
       </c>
       <c r="O9">
-        <v>0.0001849315068493151</v>
+        <v>0.001707954726293864</v>
       </c>
       <c r="P9">
-        <v>0.0001849315068493151</v>
+        <v>0.001707954726293864</v>
       </c>
       <c r="Q9">
-        <v>0.0001530185286095631</v>
+        <v>0.0001612188896106683</v>
       </c>
       <c r="R9">
-        <v>0.0001849315068493151</v>
+        <v>0.001707954726293864</v>
       </c>
       <c r="S9">
-        <v>0.0001849315068493151</v>
+        <v>0.001707954726293864</v>
       </c>
       <c r="T9">
-        <v>0.0001530185286095631</v>
+        <v>0.0001612188896106683</v>
       </c>
       <c r="U9">
-        <v>0.0001849315068493151</v>
+        <v>0.001707954726293864</v>
       </c>
       <c r="V9">
-        <v>0.0001849315068493151</v>
+        <v>0.001707954726293864</v>
       </c>
       <c r="W9">
-        <v>0.0001530185286095631</v>
+        <v>0.0001612188896106683</v>
       </c>
       <c r="X9">
-        <v>0.0001849315068493151</v>
+        <v>0.001707954726293864</v>
       </c>
       <c r="Y9">
-        <v>0.0002136034642349976</v>
+        <v>0.001307587988024648</v>
       </c>
       <c r="Z9">
-        <v>0.0001402202031142261</v>
+        <v>0.0001456871104482962</v>
       </c>
       <c r="AA9">
-        <v>0.0002136034642349976</v>
+        <v>0.001307587988024648</v>
       </c>
       <c r="AB9">
-        <v>0.0002451613829154453</v>
+        <v>0.001293297022188149</v>
       </c>
       <c r="AC9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AD9">
-        <v>0.0002451613829154453</v>
+        <v>0.001293297022188149</v>
       </c>
       <c r="AE9">
-        <v>0.0002451613829154453</v>
+        <v>0.001293297022188149</v>
       </c>
       <c r="AF9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AG9">
-        <v>0.0002451613829154453</v>
+        <v>0.001293297022188149</v>
       </c>
       <c r="AH9">
-        <v>0.0002451613829154453</v>
+        <v>0.001293297022188149</v>
       </c>
       <c r="AI9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AJ9">
-        <v>0.0002451613829154453</v>
+        <v>0.001293297022188149</v>
       </c>
       <c r="AK9">
-        <v>0.0001648236055669436</v>
+        <v>0.001135986550563039</v>
       </c>
       <c r="AL9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AM9">
-        <v>0.0001648236055669436</v>
+        <v>0.001135986550563039</v>
       </c>
       <c r="AN9">
-        <v>0.0001648236055669436</v>
+        <v>0.001135986550563039</v>
       </c>
       <c r="AO9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AP9">
-        <v>0.0001648236055669436</v>
+        <v>0.001135986550563039</v>
       </c>
       <c r="AQ9">
-        <v>0.0001849315068493151</v>
+        <v>0.001707954726293864</v>
       </c>
       <c r="AR9">
-        <v>0.0001530185286095631</v>
+        <v>0.0001612188896106683</v>
       </c>
       <c r="AS9">
-        <v>0.0001849315068493151</v>
+        <v>0.001707954726293864</v>
       </c>
       <c r="AT9">
-        <v>0.000248512888301388</v>
+        <v>0.001165164560208317</v>
       </c>
       <c r="AU9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AV9">
-        <v>0.000248512888301388</v>
+        <v>0.001165164560208317</v>
       </c>
       <c r="AW9">
-        <v>0.000248512888301388</v>
+        <v>0.001165164560208317</v>
       </c>
       <c r="AX9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AY9">
-        <v>0.000248512888301388</v>
+        <v>0.001165164560208317</v>
       </c>
       <c r="AZ9">
-        <v>0.0001648236055669436</v>
+        <v>0.001135986550563039</v>
       </c>
       <c r="BA9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="BB9">
-        <v>0.0001648236055669436</v>
+        <v>0.001135986550563039</v>
       </c>
       <c r="BC9">
-        <v>0.0001648236055669436</v>
+        <v>0.001135986550563039</v>
       </c>
       <c r="BD9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="BE9">
-        <v>0.0001648236055669436</v>
+        <v>0.001135986550563039</v>
       </c>
     </row>
     <row r="10" spans="1:57">
       <c r="A10">
-        <v>0.000235106866757617</v>
+        <v>0.04441680680005174</v>
       </c>
       <c r="B10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="C10">
-        <v>0.000235106866757617</v>
+        <v>0.04441680680005174</v>
       </c>
       <c r="D10">
-        <v>0.000235106866757617</v>
+        <v>0.04441680680005174</v>
       </c>
       <c r="E10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="F10">
-        <v>0.000235106866757617</v>
+        <v>0.04441680680005174</v>
       </c>
       <c r="G10">
-        <v>0.0001849315068493151</v>
+        <v>0.01150025399955056</v>
       </c>
       <c r="H10">
-        <v>0.0001530185286095631</v>
+        <v>0.0001612188896106683</v>
       </c>
       <c r="I10">
-        <v>0.0001849315068493151</v>
+        <v>0.01150025399955056</v>
       </c>
       <c r="J10">
-        <v>0.0002451613829154453</v>
+        <v>0.02491652076564341</v>
       </c>
       <c r="K10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="L10">
-        <v>0.0002451613829154453</v>
+        <v>0.02491652076564341</v>
       </c>
       <c r="M10">
-        <v>0.0001849315068493151</v>
+        <v>0.01150025399955056</v>
       </c>
       <c r="N10">
-        <v>0.0001530185286095631</v>
+        <v>0.0001612188896106683</v>
       </c>
       <c r="O10">
-        <v>0.0001849315068493151</v>
+        <v>0.01150025399955056</v>
       </c>
       <c r="P10">
-        <v>0.0001849315068493151</v>
+        <v>0.01150025399955056</v>
       </c>
       <c r="Q10">
-        <v>0.0001530185286095631</v>
+        <v>0.0001612188896106683</v>
       </c>
       <c r="R10">
-        <v>0.0001849315068493151</v>
+        <v>0.01150025399955056</v>
       </c>
       <c r="S10">
-        <v>0.0001849315068493151</v>
+        <v>0.01150025399955056</v>
       </c>
       <c r="T10">
-        <v>0.0001530185286095631</v>
+        <v>0.0001612188896106683</v>
       </c>
       <c r="U10">
-        <v>0.0001849315068493151</v>
+        <v>0.01150025399955056</v>
       </c>
       <c r="V10">
-        <v>0.0001849315068493151</v>
+        <v>0.01150025399955056</v>
       </c>
       <c r="W10">
-        <v>0.0001530185286095631</v>
+        <v>0.0001612188896106683</v>
       </c>
       <c r="X10">
-        <v>0.0001849315068493151</v>
+        <v>0.01150025399955056</v>
       </c>
       <c r="Y10">
-        <v>0.0002136034642349976</v>
+        <v>0.01915307147756048</v>
       </c>
       <c r="Z10">
-        <v>0.0001402202031142261</v>
+        <v>0.0001456871104482962</v>
       </c>
       <c r="AA10">
-        <v>0.0002136034642349976</v>
+        <v>0.01915307147756048</v>
       </c>
       <c r="AB10">
-        <v>0.0002451613829154453</v>
+        <v>0.02491652076564341</v>
       </c>
       <c r="AC10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AD10">
-        <v>0.0002451613829154453</v>
+        <v>0.02491652076564341</v>
       </c>
       <c r="AE10">
-        <v>0.0002451613829154453</v>
+        <v>0.02491652076564341</v>
       </c>
       <c r="AF10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AG10">
-        <v>0.0002451613829154453</v>
+        <v>0.02491652076564341</v>
       </c>
       <c r="AH10">
-        <v>0.0002451613829154453</v>
+        <v>0.02491652076564341</v>
       </c>
       <c r="AI10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AJ10">
-        <v>0.0002451613829154453</v>
+        <v>0.02491652076564341</v>
       </c>
       <c r="AK10">
-        <v>0.0001648236055669436</v>
+        <v>0.01145258164039959</v>
       </c>
       <c r="AL10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AM10">
-        <v>0.0001648236055669436</v>
+        <v>0.01145258164039959</v>
       </c>
       <c r="AN10">
-        <v>0.0001648236055669436</v>
+        <v>0.01145258164039959</v>
       </c>
       <c r="AO10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AP10">
-        <v>0.0001648236055669436</v>
+        <v>0.01145258164039959</v>
       </c>
       <c r="AQ10">
-        <v>0.0001849315068493151</v>
+        <v>0.01150025399955056</v>
       </c>
       <c r="AR10">
-        <v>0.0001530185286095631</v>
+        <v>0.0001612188896106683</v>
       </c>
       <c r="AS10">
-        <v>0.0001849315068493151</v>
+        <v>0.01150025399955056</v>
       </c>
       <c r="AT10">
-        <v>0.000248512888301388</v>
+        <v>0.01841642542084063</v>
       </c>
       <c r="AU10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AV10">
-        <v>0.000248512888301388</v>
+        <v>0.01841642542084063</v>
       </c>
       <c r="AW10">
-        <v>0.000248512888301388</v>
+        <v>0.01841642542084063</v>
       </c>
       <c r="AX10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="AY10">
-        <v>0.000248512888301388</v>
+        <v>0.01841642542084063</v>
       </c>
       <c r="AZ10">
-        <v>0.0001648236055669436</v>
+        <v>0.01145258164039959</v>
       </c>
       <c r="BA10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="BB10">
-        <v>0.0001648236055669436</v>
+        <v>0.01145258164039959</v>
       </c>
       <c r="BC10">
-        <v>0.0001648236055669436</v>
+        <v>0.01145258164039959</v>
       </c>
       <c r="BD10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="BE10">
-        <v>0.0001648236055669436</v>
+        <v>0.01145258164039959</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add stubble sim inputs for barley from Southern Dirt work. Plus tweak sgen to stop a warning (big negitive age was causing inf in back transform). Profit down 8k
</commit_message>
<xml_diff>
--- a/ExcelInputs/stubble sim.xlsx
+++ b/ExcelInputs/stubble sim.xlsx
@@ -345,22 +345,22 @@
   <sheetData>
     <row r="1" spans="1:57">
       <c r="A1">
-        <v>0.04261855969762757</v>
+        <v>0.01429408924485331</v>
       </c>
       <c r="B1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="C1">
-        <v>0.04261855969762757</v>
+        <v>0.01429408924485331</v>
       </c>
       <c r="D1">
-        <v>0.04261855969762757</v>
+        <v>0.01429408924485331</v>
       </c>
       <c r="E1">
         <v>0.0001146235521235521</v>
       </c>
       <c r="F1">
-        <v>0.04261855969762757</v>
+        <v>0.01429408924485331</v>
       </c>
       <c r="G1">
         <v>0.0441170780966807</v>
@@ -518,22 +518,22 @@
     </row>
     <row r="2" spans="1:57">
       <c r="A2">
-        <v>0.01460592263094856</v>
+        <v>0.01465413281951116</v>
       </c>
       <c r="B2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="C2">
-        <v>0.01460592263094856</v>
+        <v>0.01465413281951116</v>
       </c>
       <c r="D2">
-        <v>0.01460592263094856</v>
+        <v>0.01465413281951116</v>
       </c>
       <c r="E2">
         <v>0.0001146235521235521</v>
       </c>
       <c r="F2">
-        <v>0.01460592263094856</v>
+        <v>0.01465413281951116</v>
       </c>
       <c r="G2">
         <v>0.007592901447036864</v>
@@ -691,22 +691,22 @@
     </row>
     <row r="3" spans="1:57">
       <c r="A3">
-        <v>0.008827677126120309</v>
+        <v>0.01494561255896355</v>
       </c>
       <c r="B3">
-        <v>0.396075168941436</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="C3">
-        <v>0.008827677126120309</v>
+        <v>0.01494561255896355</v>
       </c>
       <c r="D3">
-        <v>0.008827677126120309</v>
+        <v>0.01494561255896355</v>
       </c>
       <c r="E3">
-        <v>0.396075168941436</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="F3">
-        <v>0.008827677126120309</v>
+        <v>0.01494561255896355</v>
       </c>
       <c r="G3">
         <v>0.009184016523502319</v>
@@ -721,7 +721,7 @@
         <v>0.006838682809351938</v>
       </c>
       <c r="K3">
-        <v>0.396075168941436</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="L3">
         <v>0.006838682809351938</v>
@@ -766,7 +766,7 @@
         <v>0.006869978102312557</v>
       </c>
       <c r="Z3">
-        <v>0.3501218683306678</v>
+        <v>0.2181350198675637</v>
       </c>
       <c r="AA3">
         <v>0.006869978102312557</v>
@@ -775,7 +775,7 @@
         <v>0.006838682809351938</v>
       </c>
       <c r="AC3">
-        <v>0.396075168941436</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AD3">
         <v>0.006838682809351938</v>
@@ -784,7 +784,7 @@
         <v>0.006838682809351938</v>
       </c>
       <c r="AF3">
-        <v>0.396075168941436</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AG3">
         <v>0.006838682809351938</v>
@@ -793,7 +793,7 @@
         <v>0.006838682809351938</v>
       </c>
       <c r="AI3">
-        <v>0.396075168941436</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AJ3">
         <v>0.006838682809351938</v>
@@ -802,7 +802,7 @@
         <v>0.005775549477638912</v>
       </c>
       <c r="AL3">
-        <v>0.396075168941436</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AM3">
         <v>0.005775549477638912</v>
@@ -811,7 +811,7 @@
         <v>0.005775549477638912</v>
       </c>
       <c r="AO3">
-        <v>0.396075168941436</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AP3">
         <v>0.005775549477638912</v>
@@ -829,7 +829,7 @@
         <v>0.006175684703762482</v>
       </c>
       <c r="AU3">
-        <v>0.396075168941436</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AV3">
         <v>0.006175684703762482</v>
@@ -838,7 +838,7 @@
         <v>0.006175684703762482</v>
       </c>
       <c r="AX3">
-        <v>0.396075168941436</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AY3">
         <v>0.006175684703762482</v>
@@ -847,7 +847,7 @@
         <v>0.005775549477638912</v>
       </c>
       <c r="BA3">
-        <v>0.396075168941436</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="BB3">
         <v>0.005775549477638912</v>
@@ -856,7 +856,7 @@
         <v>0.005775549477638912</v>
       </c>
       <c r="BD3">
-        <v>0.396075168941436</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="BE3">
         <v>0.005775549477638912</v>
@@ -864,22 +864,22 @@
     </row>
     <row r="4" spans="1:57">
       <c r="A4">
-        <v>0.01189379243929846</v>
+        <v>0.01183798783845969</v>
       </c>
       <c r="B4">
-        <v>0.1430970420835792</v>
+        <v>0.2603711076045888</v>
       </c>
       <c r="C4">
-        <v>0.01189379243929846</v>
+        <v>0.01183798783845969</v>
       </c>
       <c r="D4">
-        <v>0.01189379243929846</v>
+        <v>0.01183798783845969</v>
       </c>
       <c r="E4">
-        <v>0.1430970420835792</v>
+        <v>0.2603711076045888</v>
       </c>
       <c r="F4">
-        <v>0.01189379243929846</v>
+        <v>0.01183798783845969</v>
       </c>
       <c r="G4">
         <v>0.006172366134497694</v>
@@ -894,7 +894,7 @@
         <v>0.005667464598099573</v>
       </c>
       <c r="K4">
-        <v>0.1430970420835792</v>
+        <v>0.2603711076045888</v>
       </c>
       <c r="L4">
         <v>0.005667464598099573</v>
@@ -939,7 +939,7 @@
         <v>0.004890176770189002</v>
       </c>
       <c r="Z4">
-        <v>0.1428195352127116</v>
+        <v>0.1819108903863814</v>
       </c>
       <c r="AA4">
         <v>0.004890176770189002</v>
@@ -948,7 +948,7 @@
         <v>0.005667464598099573</v>
       </c>
       <c r="AC4">
-        <v>0.1430970420835792</v>
+        <v>0.2603711076045888</v>
       </c>
       <c r="AD4">
         <v>0.005667464598099573</v>
@@ -957,7 +957,7 @@
         <v>0.005667464598099573</v>
       </c>
       <c r="AF4">
-        <v>0.1430970420835792</v>
+        <v>0.2603711076045888</v>
       </c>
       <c r="AG4">
         <v>0.005667464598099573</v>
@@ -966,7 +966,7 @@
         <v>0.005667464598099573</v>
       </c>
       <c r="AI4">
-        <v>0.1430970420835792</v>
+        <v>0.2603711076045888</v>
       </c>
       <c r="AJ4">
         <v>0.005667464598099573</v>
@@ -975,7 +975,7 @@
         <v>0.002694506432213508</v>
       </c>
       <c r="AL4">
-        <v>0.1430970420835792</v>
+        <v>0.2603711076045888</v>
       </c>
       <c r="AM4">
         <v>0.002694506432213508</v>
@@ -984,7 +984,7 @@
         <v>0.002694506432213508</v>
       </c>
       <c r="AO4">
-        <v>0.1430970420835792</v>
+        <v>0.2603711076045888</v>
       </c>
       <c r="AP4">
         <v>0.002694506432213508</v>
@@ -1002,7 +1002,7 @@
         <v>0.003592021984366611</v>
       </c>
       <c r="AU4">
-        <v>0.1430970420835792</v>
+        <v>0.2603711076045888</v>
       </c>
       <c r="AV4">
         <v>0.003592021984366611</v>
@@ -1011,7 +1011,7 @@
         <v>0.003592021984366611</v>
       </c>
       <c r="AX4">
-        <v>0.1430970420835792</v>
+        <v>0.2603711076045888</v>
       </c>
       <c r="AY4">
         <v>0.003592021984366611</v>
@@ -1020,7 +1020,7 @@
         <v>0.002694506432213508</v>
       </c>
       <c r="BA4">
-        <v>0.1430970420835792</v>
+        <v>0.2603711076045888</v>
       </c>
       <c r="BB4">
         <v>0.002694506432213508</v>
@@ -1029,7 +1029,7 @@
         <v>0.002694506432213508</v>
       </c>
       <c r="BD4">
-        <v>0.1430970420835792</v>
+        <v>0.2603711076045888</v>
       </c>
       <c r="BE4">
         <v>0.002694506432213508</v>
@@ -1037,22 +1037,22 @@
     </row>
     <row r="5" spans="1:57">
       <c r="A5">
-        <v>0.007020063450574888</v>
+        <v>0.01352684868905732</v>
       </c>
       <c r="B5">
-        <v>0.1448482868644593</v>
+        <v>0.0396990417921626</v>
       </c>
       <c r="C5">
-        <v>0.007020063450574888</v>
+        <v>0.01352684868905732</v>
       </c>
       <c r="D5">
-        <v>0.007020063450574888</v>
+        <v>0.01352684868905732</v>
       </c>
       <c r="E5">
-        <v>0.1448482868644593</v>
+        <v>0.0396990417921626</v>
       </c>
       <c r="F5">
-        <v>0.007020063450574888</v>
+        <v>0.01352684868905732</v>
       </c>
       <c r="G5">
         <v>0.009108166267423327</v>
@@ -1067,7 +1067,7 @@
         <v>0.004908398109682398</v>
       </c>
       <c r="K5">
-        <v>0.1448482868644593</v>
+        <v>0.0396990417921626</v>
       </c>
       <c r="L5">
         <v>0.004908398109682398</v>
@@ -1112,7 +1112,7 @@
         <v>0.005102479196887717</v>
       </c>
       <c r="Z5">
-        <v>0.1362042619326106</v>
+        <v>0.1011545135751784</v>
       </c>
       <c r="AA5">
         <v>0.005102479196887717</v>
@@ -1121,7 +1121,7 @@
         <v>0.004908398109682398</v>
       </c>
       <c r="AC5">
-        <v>0.1448482868644593</v>
+        <v>0.0396990417921626</v>
       </c>
       <c r="AD5">
         <v>0.004908398109682398</v>
@@ -1130,7 +1130,7 @@
         <v>0.004908398109682398</v>
       </c>
       <c r="AF5">
-        <v>0.1448482868644593</v>
+        <v>0.0396990417921626</v>
       </c>
       <c r="AG5">
         <v>0.004908398109682398</v>
@@ -1139,7 +1139,7 @@
         <v>0.004908398109682398</v>
       </c>
       <c r="AI5">
-        <v>0.1448482868644593</v>
+        <v>0.0396990417921626</v>
       </c>
       <c r="AJ5">
         <v>0.004908398109682398</v>
@@ -1148,7 +1148,7 @@
         <v>0.003487797836030551</v>
       </c>
       <c r="AL5">
-        <v>0.1448482868644593</v>
+        <v>0.0396990417921626</v>
       </c>
       <c r="AM5">
         <v>0.003487797836030551</v>
@@ -1157,7 +1157,7 @@
         <v>0.003487797836030551</v>
       </c>
       <c r="AO5">
-        <v>0.1448482868644593</v>
+        <v>0.0396990417921626</v>
       </c>
       <c r="AP5">
         <v>0.003487797836030551</v>
@@ -1175,7 +1175,7 @@
         <v>0.004204509662718235</v>
       </c>
       <c r="AU5">
-        <v>0.1448482868644593</v>
+        <v>0.0396990417921626</v>
       </c>
       <c r="AV5">
         <v>0.004204509662718235</v>
@@ -1184,7 +1184,7 @@
         <v>0.004204509662718235</v>
       </c>
       <c r="AX5">
-        <v>0.1448482868644593</v>
+        <v>0.0396990417921626</v>
       </c>
       <c r="AY5">
         <v>0.004204509662718235</v>
@@ -1193,7 +1193,7 @@
         <v>0.003487797836030551</v>
       </c>
       <c r="BA5">
-        <v>0.1448482868644593</v>
+        <v>0.0396990417921626</v>
       </c>
       <c r="BB5">
         <v>0.003487797836030551</v>
@@ -1202,7 +1202,7 @@
         <v>0.003487797836030551</v>
       </c>
       <c r="BD5">
-        <v>0.1448482868644593</v>
+        <v>0.0396990417921626</v>
       </c>
       <c r="BE5">
         <v>0.003487797836030551</v>
@@ -1210,22 +1210,22 @@
     </row>
     <row r="6" spans="1:57">
       <c r="A6">
-        <v>0.006105371091459948</v>
+        <v>0.01235557501584071</v>
       </c>
       <c r="B6">
-        <v>0.08568051951151724</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="C6">
-        <v>0.006105371091459948</v>
+        <v>0.01235557501584071</v>
       </c>
       <c r="D6">
-        <v>0.006105371091459948</v>
+        <v>0.01235557501584071</v>
       </c>
       <c r="E6">
-        <v>0.08568051951151724</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="F6">
-        <v>0.006105371091459948</v>
+        <v>0.01235557501584071</v>
       </c>
       <c r="G6">
         <v>0.006328575760998325</v>
@@ -1240,7 +1240,7 @@
         <v>0.004707971756326143</v>
       </c>
       <c r="K6">
-        <v>0.08568051951151724</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="L6">
         <v>0.004707971756326143</v>
@@ -1285,7 +1285,7 @@
         <v>0.00446100092028795</v>
       </c>
       <c r="Z6">
-        <v>0.1170635261296166</v>
+        <v>0.0885415608098187</v>
       </c>
       <c r="AA6">
         <v>0.00446100092028795</v>
@@ -1294,7 +1294,7 @@
         <v>0.004707971756326143</v>
       </c>
       <c r="AC6">
-        <v>0.08568051951151724</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AD6">
         <v>0.004707971756326143</v>
@@ -1303,7 +1303,7 @@
         <v>0.004707971756326143</v>
       </c>
       <c r="AF6">
-        <v>0.08568051951151724</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AG6">
         <v>0.004707971756326143</v>
@@ -1312,7 +1312,7 @@
         <v>0.004707971756326143</v>
       </c>
       <c r="AI6">
-        <v>0.08568051951151724</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AJ6">
         <v>0.004707971756326143</v>
@@ -1321,7 +1321,7 @@
         <v>0.003033271827856376</v>
       </c>
       <c r="AL6">
-        <v>0.08568051951151724</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AM6">
         <v>0.003033271827856376</v>
@@ -1330,7 +1330,7 @@
         <v>0.003033271827856376</v>
       </c>
       <c r="AO6">
-        <v>0.08568051951151724</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AP6">
         <v>0.003033271827856376</v>
@@ -1348,7 +1348,7 @@
         <v>0.004242171977948208</v>
       </c>
       <c r="AU6">
-        <v>0.08568051951151724</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AV6">
         <v>0.004242171977948208</v>
@@ -1357,7 +1357,7 @@
         <v>0.004242171977948208</v>
       </c>
       <c r="AX6">
-        <v>0.08568051951151724</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="AY6">
         <v>0.004242171977948208</v>
@@ -1366,7 +1366,7 @@
         <v>0.003033271827856376</v>
       </c>
       <c r="BA6">
-        <v>0.08568051951151724</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="BB6">
         <v>0.003033271827856376</v>
@@ -1375,7 +1375,7 @@
         <v>0.003033271827856376</v>
       </c>
       <c r="BD6">
-        <v>0.08568051951151724</v>
+        <v>0.0001146235521235521</v>
       </c>
       <c r="BE6">
         <v>0.003033271827856376</v>
@@ -1383,22 +1383,22 @@
     </row>
     <row r="7" spans="1:57">
       <c r="A7">
-        <v>0.007792132306019362</v>
+        <v>0.009218405000433461</v>
       </c>
       <c r="B7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="C7">
-        <v>0.007792132306019362</v>
+        <v>0.009218405000433461</v>
       </c>
       <c r="D7">
-        <v>0.007792132306019362</v>
+        <v>0.009218405000433461</v>
       </c>
       <c r="E7">
         <v>0.0001146235521235521</v>
       </c>
       <c r="F7">
-        <v>0.007792132306019362</v>
+        <v>0.009218405000433461</v>
       </c>
       <c r="G7">
         <v>0.005366987015587355</v>
@@ -1556,22 +1556,22 @@
     </row>
     <row r="8" spans="1:57">
       <c r="A8">
-        <v>0.004276090778868289</v>
+        <v>0.005023519932427278</v>
       </c>
       <c r="B8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="C8">
-        <v>0.004276090778868289</v>
+        <v>0.005023519932427278</v>
       </c>
       <c r="D8">
-        <v>0.004276090778868289</v>
+        <v>0.005023519932427278</v>
       </c>
       <c r="E8">
         <v>0.0001146235521235521</v>
       </c>
       <c r="F8">
-        <v>0.004276090778868289</v>
+        <v>0.005023519932427278</v>
       </c>
       <c r="G8">
         <v>0.002197409566330036</v>
@@ -1729,22 +1729,22 @@
     </row>
     <row r="9" spans="1:57">
       <c r="A9">
-        <v>0.001677694408127644</v>
+        <v>0.002801111206686857</v>
       </c>
       <c r="B9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="C9">
-        <v>0.001677694408127644</v>
+        <v>0.002801111206686857</v>
       </c>
       <c r="D9">
-        <v>0.001677694408127644</v>
+        <v>0.002801111206686857</v>
       </c>
       <c r="E9">
         <v>0.0001146235521235521</v>
       </c>
       <c r="F9">
-        <v>0.001677694408127644</v>
+        <v>0.002801111206686857</v>
       </c>
       <c r="G9">
         <v>0.001707954726293864</v>
@@ -1902,22 +1902,22 @@
     </row>
     <row r="10" spans="1:57">
       <c r="A10">
-        <v>0.04441680680005174</v>
+        <v>0.0175989551799571</v>
       </c>
       <c r="B10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="C10">
-        <v>0.04441680680005174</v>
+        <v>0.0175989551799571</v>
       </c>
       <c r="D10">
-        <v>0.04441680680005174</v>
+        <v>0.0175989551799571</v>
       </c>
       <c r="E10">
         <v>0.0001146235521235521</v>
       </c>
       <c r="F10">
-        <v>0.04441680680005174</v>
+        <v>0.0175989551799571</v>
       </c>
       <c r="G10">
         <v>0.01150025399955056</v>

</xml_diff>